<commit_message>
Update nightly research results
</commit_message>
<xml_diff>
--- a/reports/latest_investor_report.xlsx
+++ b/reports/latest_investor_report.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YONETICI_OZETI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PORTFOY_ONERISI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ILK_20_SIRALAMA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AL_SAT_OZET" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PORTFOY_DEGISIMI" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIYASA_REJIMI" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAPER_TRADE" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="YONETICI_OZETI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PORTFOY_ONERISI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ILK_20_SIRALAMA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AL_SAT_OZET" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PORTFOY_DEGISIMI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PIYASA_REJIMI" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PAPER_TRADE" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'YONETICI_OZETI'!$A$19:$K$25</definedName>
@@ -629,7 +629,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-06-24 01:23</t>
+          <t>Son Güncelleme: 2026-06-24 05:56</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -1012,7 +1012,7 @@
         <v>0.0768720785569736</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>830.864036650928</v>
+        <v>830.8640366509281</v>
       </c>
       <c r="H21" s="8" t="n">
         <v>425.0952530103654</v>
@@ -1044,16 +1044,16 @@
         </is>
       </c>
       <c r="D22" s="7" t="n">
-        <v>0.09261351611588012</v>
+        <v>0.09261351611588006</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>9261.351611588012</v>
+        <v>9261.351611588007</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>0.0426715939840771</v>
+        <v>0.0426715939840769</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>395.1966357134618</v>
+        <v>395.1966357134597</v>
       </c>
       <c r="H22" s="8" t="n">
         <v>149.8319048735307</v>
@@ -1062,7 +1062,7 @@
         <v>136.1580975269861</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.8130455715182764</v>
+        <v>0.8130455715182726</v>
       </c>
       <c r="K22" s="9" t="inlineStr">
         <is>
@@ -1085,16 +1085,16 @@
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>0.09145120548407606</v>
+        <v>0.09145120548407609</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>9145.120548407607</v>
+        <v>9145.120548407609</v>
       </c>
       <c r="F23" s="7" t="n">
         <v>0.0433601726374674</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>396.5340057694044</v>
+        <v>396.5340057694045</v>
       </c>
       <c r="H23" s="8" t="n">
         <v>42.08914952339957</v>
@@ -1103,7 +1103,7 @@
         <v>38.0275160674077</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.7563941226758241</v>
+        <v>0.7563941226758264</v>
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-06-24 01:23</t>
+          <t>Son Güncelleme: 2026-06-24 05:56</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1560,7 +1560,7 @@
         <v>0.0213779187417526</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>0.1020952413749239</v>
+        <v>0.1020952413749238</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>377.5937136635377</v>
@@ -1842,7 +1842,7 @@
         <v>-0.0082889988742848</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>0.0426715939840771</v>
+        <v>0.0426715939840769</v>
       </c>
       <c r="G15" s="19" t="n">
         <v>0.1446541396482852</v>
@@ -1896,7 +1896,7 @@
         <v>40.34000015258789</v>
       </c>
       <c r="E16" s="19" t="n">
-        <v>-0.0573248407643312</v>
+        <v>-0.057324840764331</v>
       </c>
       <c r="F16" s="19" t="n">
         <v>0.0433601726374674</v>
@@ -1953,16 +1953,16 @@
         <v>113.1999969482422</v>
       </c>
       <c r="E17" s="22" t="n">
-        <v>-0.0669128100843053</v>
+        <v>-0.0669128100843052</v>
       </c>
       <c r="F17" s="22" t="n">
         <v>-0.0163197887030124</v>
       </c>
       <c r="G17" s="22" t="n">
-        <v>0.0289375192237391</v>
+        <v>0.0289375192237388</v>
       </c>
       <c r="H17" s="21" t="n">
-        <v>105.6254670509005</v>
+        <v>105.6254670509006</v>
       </c>
       <c r="I17" s="21" t="n">
         <v>111.3525969168652</v>
@@ -1971,7 +1971,7 @@
         <v>116.4757240360591</v>
       </c>
       <c r="K17" s="21" t="n">
-        <v>105.6254670509005</v>
+        <v>105.6254670509006</v>
       </c>
       <c r="L17" s="20" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-06-24 01:23</t>
+          <t>Son Güncelleme: 2026-06-24 05:56</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="E6" s="16" t="n">
-        <v>-0.0299835584767572</v>
+        <v>-0.0299835584767574</v>
       </c>
       <c r="F6" s="16" t="n">
         <v>0.1213361981009177</v>
@@ -2234,7 +2234,7 @@
         </is>
       </c>
       <c r="J6" s="16" t="n">
-        <v>0.0211148533864321</v>
+        <v>0.0211148533864322</v>
       </c>
       <c r="K6" s="16" t="n">
         <v>0.0213779187417526</v>
@@ -2266,7 +2266,7 @@
         <v>0.1653136531365313</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>0.8699667862938347</v>
+        <v>0.8699667862938349</v>
       </c>
       <c r="H7" s="19" t="n">
         <v>-0.0591229013786693</v>
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="J7" s="19" t="n">
-        <v>0.0310679439959384</v>
+        <v>0.0310679439959383</v>
       </c>
       <c r="K7" s="19" t="n">
         <v>0.0768720785569736</v>
@@ -2309,7 +2309,7 @@
         <v>0.1429801894918174</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>0.4539139831828924</v>
+        <v>0.4539139831828926</v>
       </c>
       <c r="H8" s="22" t="n">
         <v>-0.2081217061911366</v>
@@ -2406,7 +2406,7 @@
         </is>
       </c>
       <c r="J10" s="22" t="n">
-        <v>0.0228216736000703</v>
+        <v>0.0228216736000704</v>
       </c>
       <c r="K10" s="22" t="n">
         <v>-0.0276025019756407</v>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.1749795041904276</v>
+        <v>0.1749795041904278</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>0.106639870007295</v>
@@ -2452,7 +2452,7 @@
         <v>0.0262418217864421</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>0.0426715939840771</v>
+        <v>0.0426715939840769</v>
       </c>
     </row>
     <row r="12">
@@ -2478,7 +2478,7 @@
         <v>0.0570968227884278</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>0.4655377772831777</v>
+        <v>0.4655377772831774</v>
       </c>
       <c r="G12" s="19" t="n">
         <v>0.6648414617414236</v>
@@ -2518,10 +2518,10 @@
         </is>
       </c>
       <c r="E13" s="22" t="n">
-        <v>0.0629107694670627</v>
+        <v>0.06291076946706289</v>
       </c>
       <c r="F13" s="22" t="n">
-        <v>0.0619136826322126</v>
+        <v>0.0619136826322128</v>
       </c>
       <c r="G13" s="22" t="n">
         <v>0.1418368479304974</v>
@@ -2564,10 +2564,10 @@
         <v>0.0345423149419388</v>
       </c>
       <c r="F14" s="24" t="n">
-        <v>-0.1816940257117537</v>
+        <v>-0.1816940257117536</v>
       </c>
       <c r="G14" s="24" t="n">
-        <v>-0.0253416715336882</v>
+        <v>-0.025341671533688</v>
       </c>
       <c r="H14" s="24" t="n">
         <v>0.1964250089917667</v>
@@ -2578,7 +2578,7 @@
         </is>
       </c>
       <c r="J14" s="24" t="n">
-        <v>0.022792917168649</v>
+        <v>0.0227929171686489</v>
       </c>
       <c r="K14" s="24" t="n">
         <v>0.1212597571915075</v>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="J15" s="24" t="n">
-        <v>0.0216298884764837</v>
+        <v>0.0216298884764838</v>
       </c>
       <c r="K15" s="24" t="n">
         <v>0.0194030930076112</v>
@@ -2667,7 +2667,7 @@
         <v>0.0217920353963226</v>
       </c>
       <c r="K16" s="24" t="n">
-        <v>0.009701613552635499</v>
+        <v>0.0097016135526356</v>
       </c>
     </row>
     <row r="17">
@@ -2690,13 +2690,13 @@
         </is>
       </c>
       <c r="E17" s="24" t="n">
-        <v>0.0371797344514563</v>
+        <v>0.0371797344514566</v>
       </c>
       <c r="F17" s="24" t="n">
         <v>0.0601449391773718</v>
       </c>
       <c r="G17" s="24" t="n">
-        <v>0.2087071438141818</v>
+        <v>0.2087071438141816</v>
       </c>
       <c r="H17" s="24" t="n">
         <v>-0.2858393418307774</v>
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>-0.0921431863137641</v>
+        <v>-0.092143186313764</v>
       </c>
       <c r="F18" s="24" t="n">
         <v>-0.1285291334718965</v>
@@ -2750,7 +2750,7 @@
         </is>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.023247051091997</v>
+        <v>0.0232470510919971</v>
       </c>
       <c r="K18" s="24" t="n">
         <v>0.1002252478096075</v>
@@ -2782,7 +2782,7 @@
         <v>-0.1188034318451188</v>
       </c>
       <c r="G19" s="24" t="n">
-        <v>-0.0427112219541819</v>
+        <v>-0.042711221954182</v>
       </c>
       <c r="H19" s="24" t="n">
         <v>-0.2797685248578938</v>
@@ -2819,13 +2819,13 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>-0.1274762778640684</v>
+        <v>-0.1274762778640682</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-0.0029527296674942</v>
+        <v>-0.0029527296674941</v>
       </c>
       <c r="G20" s="24" t="n">
-        <v>0.2016607055424879</v>
+        <v>0.2016607055424881</v>
       </c>
       <c r="H20" s="24" t="n">
         <v>-0.3414386978886042</v>
@@ -2872,7 +2872,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-06-24 01:23</t>
+          <t>Son Güncelleme: 2026-06-24 05:56</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2991,7 +2991,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-06-24 01:23</t>
+          <t>Son Güncelleme: 2026-06-24 05:56</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3242,7 +3242,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-06-24 01:23</t>
+          <t>Son Güncelleme: 2026-06-24 05:56</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3266,7 +3266,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>14729.7001953125</v>
+        <v>14539.599609375</v>
       </c>
     </row>
     <row r="5">
@@ -3276,7 +3276,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>12472.33203125</v>
+        <v>12490.64252929687</v>
       </c>
     </row>
     <row r="6">
@@ -3367,7 +3367,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-06-24 01:23</t>
+          <t>Son Güncelleme: 2026-06-24 05:56</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3444,7 +3444,7 @@
         <v>837.2925543086967</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H4" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3474,7 +3474,7 @@
         <v>-988.1583320280206</v>
       </c>
       <c r="G5" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3504,7 +3504,7 @@
         <v>1673.436127495303</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H6" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3534,7 +3534,7 @@
         <v>-86.53860825758602</v>
       </c>
       <c r="G7" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H7" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3564,7 +3564,7 @@
         <v>545.7748465300665</v>
       </c>
       <c r="G8" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H8" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3594,7 +3594,7 @@
         <v>540.6591394445386</v>
       </c>
       <c r="G9" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H9" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3624,7 +3624,7 @@
         <v>626.2626262626254</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H10" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3654,7 +3654,7 @@
         <v>839.84375</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H11" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3684,7 +3684,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H12" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3714,7 +3714,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H13" s="26" t="n">
         <v>0.0748467743222782</v>
@@ -3744,7 +3744,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>2277611.882914566</v>
+        <v>2311235.193725377</v>
       </c>
       <c r="H14" s="26" t="n">
         <v>0.0748467743222782</v>

</xml_diff>